<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-07 Le cube rouge d'Amir
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-07.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre</t>
+          <t>chambre, plancher, torchon, boîte, cubes, bois, rayon, pli, porte</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Amir veut empiler des cubes rouges. La tour tombe. Il souffle, fait une pause, puis pose un cube.</t>
+          <t>Une bande rouge barre le torchon plié. Sur le pli, un éclat de torchon luit. Amir veut la tour, maintenant. Les cubes tombent. Poitrine trop vite. Sourire parti. Papa s'accroupit. Il souffle, pause. Merci vécu. Deuxième ruse : la tour semble tenir, un pied accroche, un cube glisse. Il refuse de foncer. Un éclat de torchon tient sur le pli.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil chauffe le plancher. Le bois est tiède sous les pieds. Un cube rouge brille près du lit. La poussière danse dans le rayon. On entend les pas de papa. Papa monte l'escalier. Chaque marche fait un petit bruit. Je pose un linge, Amir. Me voilà. La chambre est claire. Le cube est rouge, papa. Oui. Il brille au soleil. Les autres cubes sont dans la boîte. On ouvre la boîte ensemble ? Oui. Tous les rouges. En ce moment, Amir joue. Il empile des cubes. Les cubes sont rouges. Amir veut une tour. Une tour, papa. Tu poses un cube, tout doux ? Amir pose un cube. Puis un autre. La tour tombe. Amir sent son ventre serré. C'est trop. Je suis fâché. La tour est tombée. Tu es fâché. On souffle. On fait une pause. Amir souffle. Un grand souffle. Amir s'assoit. Il pose les mains sur ses genoux. Il souffle encore. Il fait une pause. La pause est calme. Son ventre se desserre. Je souffle. Je fais une pause. Tu as soufflé. Tu as fait une pause. Bravo, Amir. C'est calme. Tu veux reprendre un cube ? Oui. Un cube rouge. Amir reprend un cube. Il souffle. Il fait une pause. Puis il pose un cube. La tour est petite. Elle tient.</t>
+          <t>Une bande rouge barre le torchon plié. C'est de la peinture, papa ? Tu vois la bande, Amir ? Oui, elle est rouge. C'est le cube, sous le torchon. Le cube rouge ! Maman soulève le torchon d'un geste. Le cube roule vers le plancher. Il roule ! Tu le rattrapes ? Oui, papa. Amir attrape le cube à deux mains. Il est lisse. Il chauffe un peu, Amir ? Un peu, maman. Le torchon est rêche, sous les doigts. Il gratte. Tu le sens, le torchon ? Oui, maman. Sur le pli, un éclat de torchon luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point. Des pas s'arrêtent près de la porte. Me voilà. La chambre est claire. Papa pose le torchon contre le bois. Il sent le bois. Tu le sens, le bois chaud ? Oui, papa. La boîte claque, près des genoux. Toc. Tu entends le toc, Amir ? Oui, maman. Le plancher est tiède, sous les pieds. Il est chaud. Un rayon glisse sur le torchon. Il allume le pli. On ouvre la boîte ensemble ? Oui, tous les rouges. Les cubes tapent le bord de la boîte. Ils sont rouges. Tu prends un cube, Amir ? Oui, celui-là. En ce moment, Amir prend un cube. Je veux la tour, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le bois peint. Tu mets le cube dessus ? Oui, maman. Amir pose un cube trop vite. Puis un autre, trop haut. Plus haut ! La tour penche d'un coup. Les cubes tombent sur le plancher. Ça fait un bruit sec. Oh. Amir reste surpris, les mains ouvertes. Sa poitrine va trop vite. Le sourire d'Amir disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. C'est trop. L'éclat de torchon tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil chauffe le plancher. Le bois est tiède sous les pieds. Un cube rouge brille près du lit. La poussière danse dans le rayon. On entend les pas de papa. Papa monte l'escalier. Chaque marche fait un petit bruit. Je pose un linge, Amir. Me voilà. La chambre est claire. Le cube est rouge, papa. Oui. Il brille au soleil. Les autres cubes sont dans la boîte. On ouvre la boîte ensemble ? Oui. Tous les rouges. En ce moment, Amir joue. Il empile des cubes. Les cubes sont rouges. Amir veut une tour. Une tour, papa. Tu poses un cube, tout doux ? Amir pose un cube. Puis un autre. La tour tombe. Amir sent son ventre serré. C'est trop. Je suis fâché. La tour est tombée. Tu es fâché. On souffle. On fait une pause. Amir souffle. Un grand souffle. Amir s'assoit. Il pose les mains sur ses genoux. Il souffle encore. Il fait une pause. La pause est calme. Son ventre se desserre. Je souffle. Je fais une pause. Tu as soufflé. Tu as fait une pause. Bravo, Amir. C'est calme. Tu veux reprendre un cube ? Oui. Un cube rouge. Amir reprend un cube. Il souffle. Il fait une pause. Puis il pose un cube. La tour est petite. Elle tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une bande rouge barre le torchon plié. C'est de la peinture, papa ? Tu vois la bande, Amir ? Oui, elle est rouge. C'est le cube, sous le torchon. Le cube rouge ! Maman soulève le torchon d'un geste. Le cube roule vers le plancher. Il roule ! Tu le rattrapes ? Oui, papa. Amir attrape le cube à deux mains. Il est lisse. Il chauffe un peu, Amir ? Un peu, maman. Le torchon est rêche, sous les doigts. Il gratte. Tu le sens, le torchon ? Oui, maman. Sur le pli, un &lt;emphasis level="moderate"&gt;éclat de torchon&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point. Des pas s'arrêtent près de la porte. Me voilà. La chambre est claire. Papa pose le torchon contre le bois. Il sent le bois. Tu le sens, le bois chaud ? Oui, papa. La boîte claque, près des genoux. Toc. Tu entends le toc, Amir ? Oui, maman. Le plancher est tiède, sous les pieds. Il est chaud. Un rayon glisse sur le torchon. Il allume le pli. On ouvre la boîte ensemble ? Oui, tous les rouges. Les cubes tapent le bord de la boîte. Ils sont rouges. Tu prends un cube, Amir ? Oui, celui-là. En ce moment, Amir prend un cube. Je veux la tour, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le bois peint. Tu mets le cube dessus ? Oui, maman. Amir pose un cube trop vite. Puis un autre, trop haut. Plus haut ! La tour penche d'un coup. Les cubes tombent sur le plancher. Ça fait un bruit sec. Oh. Amir reste surpris, les mains ouvertes. Sa poitrine va trop vite. Le sourire d'Amir disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. C'est trop. L'éclat de torchon tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Géraldine construit une tour. Les cubes sont rouges. La tour tombe. Géraldine sent son ventre serré. Papa arrive. Papa dit : on souffle. Géraldine souffle. Un grand souffle. Papa dit : on fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Géraldine s'assoit. Elle pose les fesses au sol. Elle souffle encore. La pause est calme. Son ventre se desserre. Papa reste près d'elle. Géraldine reprend un cube. Elle souffle. Elle fait une pause. Puis elle pose un cube. Papa dit : tu as soufflé. Tu as fait une pause. Géraldine sourit.&lt;/slow&gt; [pause]</t>
+          <t>Une bande rouge barre le torchon plié. C'est de la peinture, papa ? Tu vois la bande, Amir ? Oui, elle est rouge. C'est le cube, sous le torchon. Le cube rouge ! Maman soulève le torchon d'un geste. Le cube roule vers le plancher. Il roule ! Tu le rattrapes ? Oui, papa. Amir attrape le cube à deux mains. Il est lisse. Il chauffe un peu, Amir ? Un peu, maman. Le torchon est rêche, sous les doigts. Il gratte. Tu le sens, le torchon ? Oui, maman. Sur le pli, un &lt;emphasis&gt;éclat de torchon&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point. Des pas s'arrêtent près de la porte. Me voilà. La chambre est claire. Papa pose le torchon contre le bois. Il sent le bois. Tu le sens, le bois chaud ? Oui, papa. La boîte claque, près des genoux. Toc. Tu entends le toc, Amir ? Oui, maman. Le plancher est tiède, sous les pieds. Il est chaud. Un rayon glisse sur le torchon. Il allume le pli. On ouvre la boîte ensemble ? Oui, tous les rouges. Les cubes tapent le bord de la boîte. Ils sont rouges. Tu prends un cube, Amir ? Oui, celui-là. En ce moment, Amir prend un cube. Je veux la tour, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le bois peint. Tu mets le cube dessus ? Oui, maman. Amir pose un cube trop vite. Puis un autre, trop haut. Plus haut ! La tour penche d'un coup. Les cubes tombent sur le plancher. Ça fait un bruit sec. Oh. Amir reste surpris, les mains ouvertes. Sa poitrine va trop vite. Le sourire d'Amir disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. C'est trop. L'éclat de torchon tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>éclat de torchon</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,57 +1319,86 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_tour_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le soleil chauffe le plancher.
-narrateur|Le bois est tiède sous les pieds.
-narrateur|Un cube rouge brille près du lit.
-narrateur|La poussière danse dans le rayon.
-narrateur|On entend les pas de papa.
-narrateur|Papa monte l'escalier.
-narrateur|Chaque marche fait un petit bruit.
-maman|Je pose un linge, Amir.
-papa|Me voilà. La chambre est claire.
-enfant-m|Le cube est rouge, papa.
-papa|Oui. Il brille au soleil.
-maman|Les autres cubes sont dans la boîte.
-papa|On ouvre la boîte ensemble ?
-enfant-m|Oui. Tous les rouges.
-narrateur|En ce moment, Amir joue.
-narrateur|Il empile des cubes.
-narrateur|Les cubes sont rouges.
-narrateur|Amir veut une tour.
-enfant-m|Une tour, papa.
-papa|Tu poses un cube, tout doux ?
-narrateur|Amir pose un cube.
-narrateur|Puis un autre.
-narrateur|La tour tombe.
-narrateur|Amir sent son ventre serré.
-enfant-m|C'est trop. Je suis fâché.
-papa|La tour est tombée. Tu es fâché.
-papa|On souffle.
-maman|On fait une pause.
-narrateur|Amir souffle.
-narrateur|Un grand souffle.
-narrateur|Amir s'assoit.
-narrateur|Il pose les mains sur ses genoux.
-narrateur|Il souffle encore.
-narrateur|Il fait une pause.
-narrateur|La pause est calme.
-narrateur|Son ventre se desserre.
-enfant-m|Je souffle. Je fais une pause.
-papa|Tu as soufflé. Tu as fait une pause.
-maman|Bravo, Amir. C'est calme.
-papa|Tu veux reprendre un cube ?
-enfant-m|Oui. Un cube rouge.
-narrateur|Amir reprend un cube.
-narrateur|Il souffle.
-narrateur|Il fait une pause.
-narrateur|Puis il pose un cube.
-maman|La tour est petite. Elle tient.</t>
+          <t>narrateur|Une bande rouge barre le torchon plié.
+enfant-m|C'est de la peinture, papa ?
+papa|Tu vois la bande, Amir ?
+enfant-m|Oui, elle est rouge.
+maman|C'est le cube, sous le torchon.
+enfant-m|Le cube rouge !
+narrateur|Maman soulève le torchon d'un geste.
+narrateur|Le cube roule vers le plancher.
+enfant-m|Il roule !
+papa|Tu le rattrapes ?
+enfant-m|Oui, papa.
+narrateur|Amir attrape le cube à deux mains.
+enfant-m|Il est lisse.
+maman|Il chauffe un peu, Amir ?
+enfant-m|Un peu, maman.
+narrateur|Le torchon est rêche, sous les doigts.
+enfant-m|Il gratte.
+maman|Tu le sens, le torchon ?
+enfant-m|Oui, maman.
+narrateur|Sur le pli, un éclat de torchon luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un point.
+narrateur|Des pas s'arrêtent près de la porte.
+papa|Me voilà.
+enfant-m|La chambre est claire.
+narrateur|Papa pose le torchon contre le bois.
+enfant-m|Il sent le bois.
+papa|Tu le sens, le bois chaud ?
+enfant-m|Oui, papa.
+narrateur|La boîte claque, près des genoux.
+enfant-m|Toc.
+maman|Tu entends le toc, Amir ?
+enfant-m|Oui, maman.
+narrateur|Le plancher est tiède, sous les pieds.
+enfant-m|Il est chaud.
+narrateur|Un rayon glisse sur le torchon.
+enfant-m|Il allume le pli.
+maman|On ouvre la boîte ensemble ?
+enfant-m|Oui, tous les rouges.
+narrateur|Les cubes tapent le bord de la boîte.
+enfant-m|Ils sont rouges.
+papa|Tu prends un cube, Amir ?
+enfant-m|Oui, celui-là.
+narrateur|En ce moment, Amir prend un cube.
+enfant-m|Je veux la tour, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Les mains serrent le bois peint.
+maman|Tu mets le cube dessus ?
+enfant-m|Oui, maman.
+narrateur|Amir pose un cube trop vite.
+narrateur|Puis un autre, trop haut.
+enfant-m|Plus haut !
+narrateur|La tour penche d'un coup.
+narrateur|Les cubes tombent sur le plancher.
+narrateur|Ça fait un bruit sec.
+enfant-m|Oh.
+narrateur|Amir reste surpris, les mains ouvertes.
+narrateur|Sa poitrine va trop vite.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois les cubes, Amir ?
+enfant-m|Oui, papa.
+maman|Tes mains sont chaudes, Amir ?
+enfant-m|Un peu, maman.
+enfant-m|C'est trop.
+narrateur|L'éclat de torchon tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1406,12 +1435,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>La tour tombe. Que fait Amir ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La tour tombe. Que fait &lt;emphasis level="moderate"&gt;Amir&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;La tour tombe. Que fait Géraldine ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;La tour tombe. Que fait &lt;emphasis&gt;Amir&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1421,7 +1450,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>souffler | elle souffle | pause | une pause | s'asseoir</t>
+          <t>souffler | il souffle | pause | une pause | s'asseoir</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1436,7 +1465,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle souffle. Elle s'assoit. Que fait-elle ?</t>
+          <t>Il souffle. Il s'assoit. Que fait-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1474,7 +1503,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1485,7 +1514,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1500,34 +1529,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Amir</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1542,7 +1575,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1552,7 +1585,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=la_tour_tombe_que_fait_amir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1585,17 +1618,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Amir a soufflé. Il a fait une pause. Le linge est plié. Je reste près de toi. Le soleil est encore sur le plancher. Le bois est chaud, papa. Oui. On reprend un cube, tout doux. Un cube glisse encore. Je souffle. Je fais une pause. Oui. On souffle. On fait une pause. Tu t'assois. Tu souffles. Amir s'assoit. Il souffle. Un grand souffle. Il fait une pause. Bravo. Tu as repris. La tour est petite. Elle tient. C'est bien.</t>
+          <t>Amir veut empiler, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre. Les mots se bousculent dans sa bouche. Trop vite. Amir avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe les cubes, un instant. Il écoute la chambre. Fff. Amir souffle une fois. Il souffle une deuxième fois. Il s'assoit près de la boîte. Ses mains se posent sur ses genoux. Il fait une pause. La poitrine ralentit un peu. Tu restes un peu, Amir ? Oui, papa. Merci, Amir. Papa reste à la même hauteur. Le bois colle un peu, sous les doigts. Il est tiède. Amir reprend un cube, sans se presser. Il le pose sur un autre. Tu le vois, le cube ? Oui, papa. La tour a deux cubes. Elle tient ! La tour est petite, Amir ? Oui, papa. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Le rayon touche le pli ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Amir a soufflé. Il a fait une pause. Le linge est plié. Je reste près de toi. Le soleil est encore sur le plancher. Le bois est chaud, papa. Oui. On reprend un cube, tout doux. Un cube glisse encore. Je souffle. Je fais une pause. Oui. On souffle. On fait une pause. Tu t'assois. Tu souffles. Amir s'assoit. Il souffle. Un grand souffle. Il fait une pause. Bravo. Tu as repris. La tour est petite. Elle tient. C'est bien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut empiler, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre. Les mots se bousculent dans sa bouche. Trop vite. Amir avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe les cubes, un instant. Il écoute la chambre. Fff. Amir &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt; une fois. Il souffle une deuxième fois. Il s'assoit près de la boîte. Ses mains se posent sur ses genoux. Il fait une pause. La poitrine ralentit un peu. Tu restes un peu, Amir ? Oui, papa. Merci, Amir. Papa reste à la même hauteur. Le bois colle un peu, sous les doigts. Il est tiède. Amir reprend un cube, sans se presser. Il le pose sur un autre. Tu le vois, le cube ? Oui, papa. La tour a deux cubes. Elle tient ! La tour est petite, Amir ? Oui, papa. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Le rayon touche le pli ? Oui, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Géraldine a soufflé. Elle a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Papa était là.&lt;/slow&gt; [pause]</t>
+          <t>Amir veut empiler, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre. Les mots se bousculent dans sa bouche. Trop vite. Amir avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe les cubes, un instant. Il écoute la chambre. Fff. Amir &lt;emphasis&gt;souffle&lt;/emphasis&gt; une fois. Il souffle une deuxième fois. Il s'assoit près de la boîte. Ses mains se posent sur ses genoux. Il fait une pause. La poitrine ralentit un peu. Tu restes un peu, Amir ? Oui, papa. Merci, Amir. Papa reste à la même hauteur. Le bois colle un peu, sous les doigts. Il est tiède. Amir reprend un cube, sans se presser. Il le pose sur un autre. Tu le vois, le cube ? Oui, papa. La tour a deux cubes. Elle tient ! La tour est petite, Amir ? Oui, papa. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près des cubes ? Oui. Le rayon touche le pli ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,18 +1675,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1676,30 +1709,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1708,10 +1741,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,33 +1753,53 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_souffle_il_fait_une_pause; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Amir a soufflé.
-narrateur|Il a fait une pause.
-maman|Le linge est plié.
-maman|Je reste près de toi.
-papa|Le soleil est encore sur le plancher.
-enfant-m|Le bois est chaud, papa.
-papa|Oui. On reprend un cube, tout doux.
-narrateur|Un cube glisse encore.
-enfant-m|Je souffle. Je fais une pause.
-papa|Oui. On souffle. On fait une pause.
-maman|Tu t'assois. Tu souffles.
-narrateur|Amir s'assoit.
-narrateur|Il souffle.
-narrateur|Un grand souffle.
+          <t>narrateur|Amir veut empiler, tout de suite.
+enfant-m|Je mets tout, maintenant !
+narrateur|Les cubes restent par terre.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Trop vite.
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe les cubes, un instant.
+narrateur|Il écoute la chambre.
+enfant-m|Fff.
+narrateur|Amir souffle une fois.
+narrateur|Il souffle une deuxième fois.
+narrateur|Il s'assoit près de la boîte.
+narrateur|Ses mains se posent sur ses genoux.
 narrateur|Il fait une pause.
-papa|Bravo. Tu as repris.
-enfant-m|La tour est petite.
-maman|Elle tient. C'est bien.</t>
+narrateur|La poitrine ralentit un peu.
+papa|Tu restes un peu, Amir ?
+enfant-m|Oui, papa.
+papa|Merci, Amir.
+narrateur|Papa reste à la même hauteur.
+maman|Le bois colle un peu, sous les doigts.
+enfant-m|Il est tiède.
+narrateur|Amir reprend un cube, sans se presser.
+narrateur|Il le pose sur un autre.
+papa|Tu le vois, le cube ?
+enfant-m|Oui, papa.
+narrateur|La tour a deux cubes.
+enfant-m|Elle tient !
+papa|La tour est petite, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près des cubes ?
+enfant-m|Oui.
+maman|Le rayon touche le pli ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1778,17 +1831,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Amir pose un cube. Le soleil touche encore le plancher. Elle tient, papa. Oui. Tu as fini de poser tes cubes ? Oui. On range la boîte ensemble ? La boîte. Puis le linge. Amir pose un cube dans la boîte. Le couvercle fait un petit bruit. Le linge est prêt. Tu viens ? Oui, maman. Le cube rouge brille encore. La chambre est calme.</t>
+          <t>Maman pousse la boîte près du plancher. Elle est un peu sèche. La tour, maintenant ! La petite tour semble tenir. Elle tient ! Amir prend trop de cubes, tout de suite. Plus haut, maintenant ! Un pied accroche le torchon. Un cube glisse au bas. Il glisse ! La tour penche, puis semble tenir. Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la tour, un instant. Il écoute la chambre, près des cubes. Sur le pli, un éclat de torchon luit. Là, sur le pli. Amir souffle une fois. Il fait une pause, assis un moment. Fff. On tient le cube ? Oui, papa. Le cube sent le bois chaud. Amir pose le cube, sans se presser. La tour se redresse. Poumf. Le bois est tiède, Amir ? Un peu. Il pose un autre cube, au milieu. Un rayon passe sur le pli. Il allume le point. Tu vois le point, Amir ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. On reste ici, Amir ? Oui. La boîte reste ouverte, près de lui. Elle sent le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Amir pose un cube. Le soleil touche encore le plancher. Elle tient, papa. Oui. Tu as fini de poser tes cubes ? Oui. On range la boîte ensemble ? La boîte. Puis le linge. Amir pose un cube dans la boîte. Le couvercle fait un petit bruit. Le linge est prêt. Tu viens ? Oui, maman. Le cube rouge brille encore. La chambre est calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse la boîte près du plancher. Elle est un peu sèche. La tour, maintenant ! La petite tour semble tenir. Elle tient ! Amir prend trop de cubes, tout de suite. Plus haut, maintenant ! Un pied accroche le torchon. Un cube glisse au bas. Il glisse ! La tour penche, puis semble tenir. Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la tour, un instant. Il écoute la chambre, près des cubes. Sur le pli, un &lt;emphasis level="moderate"&gt;éclat de torchon&lt;/emphasis&gt; luit. Là, sur le pli. Amir souffle une fois. Il fait une pause, assis un moment. Fff. On tient le cube ? Oui, papa. Le cube sent le bois chaud. Amir pose le cube, sans se presser. La tour se redresse. Poumf. Le bois est tiède, Amir ? Un peu. Il pose un autre cube, au milieu. Un rayon passe sur le pli. Il allume le point. Tu vois le point, Amir ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. On reste ici, Amir ? Oui. La boîte reste ouverte, près de lui. Elle sent le bois.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Géraldine pose un cube. La tour est petite.&lt;/slow&gt; [pause]</t>
+          <t>Maman pousse la boîte près du plancher. Elle est un peu sèche. La tour, maintenant ! La petite tour semble tenir. Elle tient ! Amir prend trop de cubes, tout de suite. Plus haut, maintenant ! Un pied accroche le torchon. Un cube glisse au bas. Il glisse ! La tour penche, puis semble tenir. Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la tour, un instant. Il écoute la chambre, près des cubes. Sur le pli, un &lt;emphasis&gt;éclat de torchon&lt;/emphasis&gt; luit. Là, sur le pli. Amir souffle une fois. Il fait une pause, assis un moment. Fff. On tient le cube ? Oui, papa. Le cube sent le bois chaud. Amir pose le cube, sans se presser. La tour se redresse. Poumf. Le bois est tiède, Amir ? Un peu. Il pose un autre cube, au milieu. Un rayon passe sur le pli. Il allume le point. Tu vois le point, Amir ? Oui, papa. Les cubes tiennent, l'un sur l'autre. C'est plus facile. On reste ici, Amir ? Oui. La boîte reste ouverte, près de lui. Elle sent le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,18 +1888,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,28 +1920,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de torchon</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1954,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1909,24 +1966,62 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=la_tour_semble_tenir_un_cube_glisse; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Amir pose un cube.
-narrateur|Le soleil touche encore le plancher.
-enfant-m|Elle tient, papa.
-papa|Oui. Tu as fini de poser tes cubes ?
+          <t>narrateur|Maman pousse la boîte près du plancher.
+narrateur|Elle est un peu sèche.
+enfant-m|La tour, maintenant !
+narrateur|La petite tour semble tenir.
+enfant-m|Elle tient !
+narrateur|Amir prend trop de cubes, tout de suite.
+enfant-m|Plus haut, maintenant !
+narrateur|Un pied accroche le torchon.
+narrateur|Un cube glisse au bas.
+enfant-m|Il glisse !
+narrateur|La tour penche, puis semble tenir.
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la tour, un instant.
+narrateur|Il écoute la chambre, près des cubes.
+narrateur|Sur le pli, un éclat de torchon luit.
+enfant-m|Là, sur le pli.
+narrateur|Amir souffle une fois.
+narrateur|Il fait une pause, assis un moment.
+enfant-m|Fff.
+papa|On tient le cube ?
+enfant-m|Oui, papa.
+narrateur|Le cube sent le bois chaud.
+narrateur|Amir pose le cube, sans se presser.
+narrateur|La tour se redresse.
+enfant-m|Poumf.
+maman|Le bois est tiède, Amir ?
+enfant-m|Un peu.
+narrateur|Il pose un autre cube, au milieu.
+maman|Un rayon passe sur le pli.
+enfant-m|Il allume le point.
+papa|Tu vois le point, Amir ?
+enfant-m|Oui, papa.
+narrateur|Les cubes tiennent, l'un sur l'autre.
+enfant-m|C'est plus facile.
+papa|On reste ici, Amir ?
 enfant-m|Oui.
-papa|On range la boîte ensemble ?
-enfant-m|La boîte. Puis le linge.
-narrateur|Amir pose un cube dans la boîte.
-narrateur|Le couvercle fait un petit bruit.
-maman|Le linge est prêt. Tu viens ?
-enfant-m|Oui, maman.
-narrateur|Le cube rouge brille encore.
-narrateur|La chambre est calme.</t>
+narrateur|La boîte reste ouverte, près de lui.
+enfant-m|Elle sent le bois.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2048,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Amir. Ta tour est petite. Elle tient.</t>
+          <t>Ils restent près de la boîte. Maman lisse un coin du torchon. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près du torchon. On est bien, ici. Amir tapote le pli du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. La tour est restée, Amir. Oui, avec les cubes. Ça sent le bois, un peu tiède. Et le torchon, maman. Oui, dans l'air. La tour reste près de la boîte. Un éclat de torchon tient sur le pli.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Amir. Ta tour est petite. Elle tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la boîte. Maman lisse un coin du torchon. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près du torchon. On est bien, ici. Amir tapote le pli du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. La tour est restée, Amir. Oui, avec les cubes. Ça sent le bois, un peu tiède. Et le torchon, maman. Oui, dans l'air. La tour reste près de la boîte. Un &lt;emphasis level="moderate"&gt;éclat de torchon&lt;/emphasis&gt; tient sur le pli.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la boîte. Maman lisse un coin du torchon. Les cubes sont tombés, papa. Tu l'as vu, toi ? Oui, près du torchon. On est bien, ici. Amir tapote le pli du doigt. Il a une trace de doigt. Tu la vois, la trace ? Oui, maman. La tour est restée, Amir. Oui, avec les cubes. Ça sent le bois, un peu tiède. Et le torchon, maman. Oui, dans l'air. La tour reste près de la boîte. Un &lt;emphasis&gt;éclat de torchon&lt;/emphasis&gt; tient sur le pli.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,7 +2105,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2018,7 +2113,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2030,12 +2125,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,14 +2139,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de torchon</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2063,11 +2162,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,26 +2175,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_pli; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai soufflé. J'ai fait une pause.
-papa|Bravo, Amir.
-maman|Ta tour est petite. Elle tient.</t>
+          <t>narrateur|Ils restent près de la boîte.
+narrateur|Maman lisse un coin du torchon.
+enfant-m|Les cubes sont tombés, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près du torchon.
+maman|On est bien, ici.
+narrateur|Amir tapote le pli du doigt.
+enfant-m|Il a une trace de doigt.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La tour est restée, Amir.
+enfant-m|Oui, avec les cubes.
+narrateur|Ça sent le bois, un peu tiède.
+enfant-m|Et le torchon, maman.
+maman|Oui, dans l'air.
+narrateur|La tour reste près de la boîte.
+narrateur|Un éclat de torchon tient sur le pli.</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2180,6 +2297,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>